<commit_message>
Brechas lote 2: recuperación ante desastres con paquete completo y RPO/RTO medidos
- NFR-07: paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas que verifica filas, huellas y cadena de auditoría y mide el tiempo; orden restaurar-paquete para un servidor nuevo (migración 0034)
- NFR-04: cinco escenarios con objetivos RPO/RTO frente a lo medido, en Preservación › Configuración
- RF-OPS-001: copia completa descargable fuera del servidor; un archivo faltante no bloquea el paquete y alerta
- RF-GOV-001 y NFR-05 fuera de alcance; matriz y documento de cierres actualizados

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -61,7 +61,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,7 +71,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -533,128 +533,108 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NO CUMPLE</t>
+          <t>NO APLICA</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NO EXISTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>17</v>
-      </c>
+          <t>Casos de prueba (12)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Casos de prueba (12)</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>CUMPLE</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>11</v>
-      </c>
+          <t>Entidades RiC-CM (19)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Entidades RiC-CM (19)</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr"/>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>17</v>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>2</v>
+          <t>Perfil AGN v1.4 (57 correspondencias)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Cubierto: 47, Parcial: 7, Ausente: 2, No adoptado (decisión): 1</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Códigos citados por el AGN que no corresponden a RiC</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>39</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Perfil AGN v1.4 (57 correspondencias)</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Cubierto: 47, Parcial: 7, Ausente: 2, No adoptado (decisión): 1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Códigos citados por el AGN que no corresponden a RiC</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
           <t>Erratas del esquema documentadas</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>13</v>
       </c>
     </row>
@@ -5493,12 +5473,12 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>NO APLICA</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>El 'fondo' (RecursoDocumental nivel=fondo, app/models/recurso_documental.py:28,41) acota datos vía fondo_id en instanciaciones/vocabulario (app/models/instanciacion.py:34). No hay modelo Organización ni asignación usuario↔fondo; permisos por módulo, no por fondo (app/core/permisos.py:84-91). docker-compose.yml:2 'una instancia por entidad'.</t>
+          <t>[Decisión] Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto. || El 'fondo' (RecursoDocumental nivel=fondo, app/models/recurso_documental.py:28,41) acota datos vía fondo_id en instanciaciones/vocabulario (app/models/instanciacion.py:34). No hay modelo Organización ni asignación usuario↔fondo; permisos por módulo, no por fondo (app/core/permisos.py:84-91). docker-compose.yml:2 'una instancia por entidad'.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -5509,7 +5489,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>No existe separación de datos entre organizaciones ni restricción de acceso por fondo: cualquier usuario con permiso de módulo ve todos los fondos.</t>
+          <t>Fuera de alcance. Riesgo residual: Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
         </is>
       </c>
     </row>
@@ -5649,7 +5629,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1] TOTP RFC 6238 con códigos de respaldo y obligatoriedad por rol: app/core/doble_factor.py, app/routers/auth.py (/login/segundo-factor, /perfil/doble-factor/*, /roles/{clave}/doble-factor, /usuarios/{id}/doble-factor/restablecer), migración 0033; tests/test_brechas_lote1.py (vectores RFC, ingreso en dos pasos, rol obligatorio, restablecimiento). || Auditoría inicial: Sin rastro de MFA/TOTP/WebAuthn en app/, frontend/src ni requirements.txt; login solo correo+contraseña (app/routers/auth.py:195).</t>
+          <t>[Lote 1] TOTP RFC 6238 con códigos de respaldo y obligatoriedad por rol: app/core/doble_factor.py, app/routers/auth.py (/login/segundo-factor, /perfil/doble-factor/*, /roles/{clave}/doble-factor, /usuarios/{id}/doble-factor/restablecer), migración 0033; tests/test_brechas_lote1.py (vectores RFC, ingreso en dos pasos, rol obligatorio, restablecimiento). || Sin rastro de MFA/TOTP/WebAuthn en app/, frontend/src ni requirements.txt; login solo correo+contraseña (app/routers/auth.py:195).</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -5842,7 +5822,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -5895,7 +5875,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -5948,7 +5928,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -6001,7 +5981,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -6308,7 +6288,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -6606,7 +6586,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -6659,7 +6639,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -6713,7 +6693,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G26" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -7211,7 +7191,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G36" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -7320,7 +7300,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1] Cadena de huellas SHA-256 calculada por disparador (migración 0032); verificar_cadena y GET /api/auditoria/cadena; sello guardado en la revisión semanal; tests/test_brechas_lote1.py (alterar y borrar con el disparador desactivado). || Auditoría inicial: Disparadores BEFORE UPDATE/DELETE/TRUNCATE en registro_auditoria (alembic/versions/0001_autenticacion_y_auditoria.py:93-109); sin rutas de edición; lectura por permiso propia/todo (app/core/permisos.py:80-89). Pruebas: tests/test_autenticacion.py::test_la_auditoria_no_se_puede_modificar_ni_borrar, tests/test_auditoria.py::test_ningun_evento_se_edita_ni_se_borra_por_ninguna_ruta. Sin encadenamiento de hashes ni sellado externo; el dueño de la BD puede desactivar el trigger.</t>
+          <t>[Lote 1] Cadena de huellas SHA-256 calculada por disparador (migración 0032); verificar_cadena y GET /api/auditoria/cadena; sello guardado en la revisión semanal; tests/test_brechas_lote1.py (alterar y borrar con el disparador desactivado). || Disparadores BEFORE UPDATE/DELETE/TRUNCATE en registro_auditoria (alembic/versions/0001_autenticacion_y_auditoria.py:93-109); sin rutas de edición; lectura por permiso propia/todo (app/core/permisos.py:80-89). Pruebas: tests/test_autenticacion.py::test_la_auditoria_no_se_puede_modificar_ni_borrar, tests/test_auditoria.py::test_ningun_evento_se_edita_ni_se_borra_por_ninguna_ruta. Sin encadenamiento de hashes ni sellado externo; el dueño de la BD puede desactivar el trigger.</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -7419,14 +7399,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G40" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1 (avanza)] /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). || Auditoría inicial: Respaldo pg_dump con SHA-256 y simulacro de restauración en BD efímera (app/servicios/respaldo.py:92-205; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella); /api/salud devuelve {'estado':'ok'} sin comprobar BD (app/main.py:84-86); logging.basicConfig a stdout (app/main.py:17); sin métricas; sin healthcheck del servicio web en docker-compose.yml.</t>
+          <t>[Lote 2 (avanza)] Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO. || [Lote 1 (avanza)] /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). || Respaldo pg_dump con SHA-256 y simulacro de restauración en BD efímera (app/servicios/respaldo.py:92-205; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella); /api/salud devuelve {'estado':'ok'} sin comprobar BD (app/main.py:84-86); logging.basicConfig a stdout (app/main.py:17); sin métricas; sin healthcheck del servicio web en docker-compose.yml.</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -7437,7 +7417,7 @@
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Faltan métricas, health check real (BD, almacenamiento, trabajador) y respaldo de los archivos del almacén (solo segunda copia en el mismo disco). Avance del Lote 1 (avanza): /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). Pendiente: Faltan métricas y el respaldo del almacén fuera del servidor (lote 2).</t>
+          <t>Faltan métricas, health check real (BD, almacenamiento, trabajador) y respaldo de los archivos del almacén (solo segunda copia en el mismo disco). Avance del Lote 1 (avanza): /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). Pendiente: Faltan métricas y el respaldo del almacén fuera del servidor (lote 2). Avance del Lote 2 (avanza): Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO. Pendiente: Solo faltan métricas.</t>
         </is>
       </c>
     </row>
@@ -7472,14 +7452,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1 (avanza)] Segundo factor y auditoría encadenada. || Auditoría inicial: bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
+          <t>[Lote 1 (avanza)] Segundo factor y auditoría encadenada. || bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -7623,14 +7603,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G44" s="6" t="inlineStr">
-        <is>
-          <t>NO EXISTE</t>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>No se encontró definición de RPO/RTO ni escenarios de disponibilidad en documentacion/ ni en código (grep RPO/RTO/'punto de recuperación' sin resultados). Despliegue de una sola instancia en un Droplet de 2 GB (app/main.py:2-4; deploy.yml).</t>
+          <t>[Lote 2] Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido. || No se encontró definición de RPO/RTO ni escenarios de disponibilidad en documentacion/ ni en código (grep RPO/RTO/'punto de recuperación' sin resultados). Despliegue de una sola instancia en un Droplet de 2 GB (app/main.py:2-4; deploy.yml).</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -7641,7 +7621,7 @@
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>No hay objetivos de RPO/RTO por escenario ni arquitectura de disponibilidad asociada.</t>
+          <t>Cerrada en el Lote 2. Riesgo residual: El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
         </is>
       </c>
     </row>
@@ -7676,14 +7656,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>NO CUMPLE</t>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Un solo proceso uvicorn sin workers (docker-entrypoint.sh:45), almacenamiento en disco local (app/servicios/almacen.py), trabajador único que sondea la BD (app/trabajador.py), segunda copia en el mismo disco (docker-compose.yml comentarios de volúmenes). Solo tope de 300 nodos en grafo (app/servicios/grafo.py:40).</t>
+          <t>[Decisión] Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor. || Un solo proceso uvicorn sin workers (docker-entrypoint.sh:45), almacenamiento en disco local (app/servicios/almacen.py), trabajador único que sondea la BD (app/trabajador.py), segunda copia en el mismo disco (docker-compose.yml comentarios de volúmenes). Solo tope de 300 nodos en grafo (app/servicios/grafo.py:40).</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -7694,7 +7674,7 @@
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>La arquitectura no escala horizontalmente ni separa almacenamiento de objetos.</t>
+          <t>Fuera de alcance. Riesgo residual: Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>
       </c>
     </row>
@@ -7729,7 +7709,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G46" s="4" t="inlineStr">
+      <c r="G46" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -7782,14 +7762,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Restauración probada de la BD en base efímera (app/servicios/respaldo.py:128-192; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella, ::test_un_volcado_alterado_hace_fallar_el_simulacro_con_alerta) y de archivos desde segunda copia (tests/test_preservacion_oais.py::test_alteracion_de_la_primaria_se_restaura_desde_la_segunda_copia). No hay prueba de recuperación completa (BD + almacén) en otro servidor.</t>
+          <t>[Lote 2] Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py. || Restauración probada de la BD en base efímera (app/servicios/respaldo.py:128-192; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella, ::test_un_volcado_alterado_hace_fallar_el_simulacro_con_alerta) y de archivos desde segunda copia (tests/test_preservacion_oais.py::test_alteracion_de_la_primaria_se_restaura_desde_la_segunda_copia). No hay prueba de recuperación completa (BD + almacén) en otro servidor.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -7800,7 +7780,7 @@
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>No se ha probado la recuperación integral del sistema (base + archivos + configuración) en un entorno nuevo.</t>
+          <t>Cerrada en el Lote 2. Riesgo residual: El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
         </is>
       </c>
     </row>
@@ -7933,14 +7913,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G50" s="4" t="inlineStr">
+      <c r="G50" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1 (avanza)] /api/salud consultable sin sesión por un monitor externo gratuito. || Auditoría inicial: Panel de alertas en aplicación (app/routers/alertas.py; app/models/alerta.py) para integridad, respaldos, formatos; logs stdout (app/main.py:17); health check trivial /api/salud (app/main.py:84). Sin métricas, sin alertas externas (correo/pager) ni logs estructurados.</t>
+          <t>[Lote 1 (avanza)] /api/salud consultable sin sesión por un monitor externo gratuito. || Panel de alertas en aplicación (app/routers/alertas.py; app/models/alerta.py) para integridad, respaldos, formatos; logs stdout (app/main.py:17); health check trivial /api/salud (app/main.py:84). Sin métricas, sin alertas externas (correo/pager) ni logs estructurados.</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -7986,7 +7966,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G51" s="4" t="inlineStr">
+      <c r="G51" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -8039,7 +8019,7 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="G52" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -8073,7 +8053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8191,7 +8171,7 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -8223,7 +8203,7 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -8255,7 +8235,7 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -8273,6 +8253,166 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Faltan CSP/HSTS, quitar la caída a HTTP y el restablecimiento de la contraseña del administrador en cada despliegue (lote 3).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>NFR-04</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>NO EXISTE</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Lote 2</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>NFR-07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Lote 2</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>RF-OPS-001</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Lote 2 (avanza)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Solo faltan métricas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>RF-GOV-001</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>NFR-05</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>NO CUMPLE</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>
       </c>
     </row>
@@ -9017,7 +9157,7 @@
           <t>Evento.</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -9071,7 +9211,7 @@
           <t>Regla.</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -9688,14 +9828,14 @@
           <t>Restaurar y comprobar integridad.</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella (BD en base efímera, compara conteos y huella de fijeza); tests/test_preservacion_oais.py::test_alteracion_de_la_primaria_se_restaura_desde_la_segunda_copia. Falta restauración integral BD+almacén en entorno nuevo.</t>
+          <t>[Lote 2] tests/test_brechas_lote2.py::test_paquete_completo_se_restaura_entero_y_mide_el_tiempo y ::test_un_archivo_alterado_en_el_paquete_hace_fallar_la_restauracion (base + archivos + auditoría).</t>
         </is>
       </c>
     </row>
@@ -9946,24 +10086,20 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>NO APLICA</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>El 'fondo' (RecursoDocumental nivel=fondo, app/models/recurso_documental.py:28,41) acota datos vía fondo_id en instanciaciones/vocabulario (app/models/instanciacion.py:34). No hay modelo Organización ni asignación usuario↔fondo; permisos por módulo, no por fondo (app/core/permisos.py:84-91). docker-compose.yml:2 'una instancia por entidad'.</t>
+          <t>[Decisión] Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto. || El 'fondo' (RecursoDocumental nivel=fondo, app/models/recurso_documental.py:28,41) acota datos vía fondo_id en instanciaciones/vocabulario (app/models/instanciacion.py:34). No hay modelo Organización ni asignación usuario↔fondo; permisos por módulo, no por fondo (app/core/permisos.py:84-91). docker-compose.yml:2 'una instancia por entidad'.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>No existe separación de datos entre organizaciones ni restricción de acceso por fondo: cualquier usuario con permiso de módulo ve todos los fondos.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Añadir entidad Organización/espacio y tabla usuario_fondo, y filtrar cada consulta por los fondos autorizados del actor en una dependencia común.</t>
-        </is>
-      </c>
+          <t>Fuera de alcance. Riesgo residual: Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -10048,7 +10184,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1] TOTP RFC 6238 con códigos de respaldo y obligatoriedad por rol: app/core/doble_factor.py, app/routers/auth.py (/login/segundo-factor, /perfil/doble-factor/*, /roles/{clave}/doble-factor, /usuarios/{id}/doble-factor/restablecer), migración 0033; tests/test_brechas_lote1.py (vectores RFC, ingreso en dos pasos, rol obligatorio, restablecimiento). || Auditoría inicial: Sin rastro de MFA/TOTP/WebAuthn en app/, frontend/src ni requirements.txt; login solo correo+contraseña (app/routers/auth.py:195).</t>
+          <t>[Lote 1] TOTP RFC 6238 con códigos de respaldo y obligatoriedad por rol: app/core/doble_factor.py, app/routers/auth.py (/login/segundo-factor, /perfil/doble-factor/*, /roles/{clave}/doble-factor, /usuarios/{id}/doble-factor/restablecer), migración 0033; tests/test_brechas_lote1.py (vectores RFC, ingreso en dos pasos, rol obligatorio, restablecimiento). || Sin rastro de MFA/TOTP/WebAuthn en app/, frontend/src ni requirements.txt; login solo correo+contraseña (app/routers/auth.py:195).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -10161,7 +10297,7 @@
           <t>RF-OCR-001</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10204,7 +10340,7 @@
           <t>RF-OCR-002</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10247,7 +10383,7 @@
           <t>RF-RIC-001</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10290,7 +10426,7 @@
           <t>RF-RIC-002</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10468,7 +10604,7 @@
           <t>RF-AI-002</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10646,7 +10782,7 @@
           <t>RF-SEARCH-001</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10689,7 +10825,7 @@
           <t>RF-SEARCH-002</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -10732,7 +10868,7 @@
           <t>RF-PRES-001</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -11018,7 +11154,7 @@
           <t>RF-INT-003</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
@@ -11095,7 +11231,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1] Cadena de huellas SHA-256 calculada por disparador (migración 0032); verificar_cadena y GET /api/auditoria/cadena; sello guardado en la revisión semanal; tests/test_brechas_lote1.py (alterar y borrar con el disparador desactivado). || Auditoría inicial: Disparadores BEFORE UPDATE/DELETE/TRUNCATE en registro_auditoria (alembic/versions/0001_autenticacion_y_auditoria.py:93-109); sin rutas de edición; lectura por permiso propia/todo (app/core/permisos.py:80-89). Pruebas: tests/test_autenticacion.py::test_la_auditoria_no_se_puede_modificar_ni_borrar, tests/test_auditoria.py::test_ningun_evento_se_edita_ni_se_borra_por_ninguna_ruta. Sin encadenamiento de hashes ni sellado externo; el dueño de la BD puede desactivar el trigger.</t>
+          <t>[Lote 1] Cadena de huellas SHA-256 calculada por disparador (migración 0032); verificar_cadena y GET /api/auditoria/cadena; sello guardado en la revisión semanal; tests/test_brechas_lote1.py (alterar y borrar con el disparador desactivado). || Disparadores BEFORE UPDATE/DELETE/TRUNCATE en registro_auditoria (alembic/versions/0001_autenticacion_y_auditoria.py:93-109); sin rutas de edición; lectura por permiso propia/todo (app/core/permisos.py:80-89). Pruebas: tests/test_autenticacion.py::test_la_auditoria_no_se_puede_modificar_ni_borrar, tests/test_auditoria.py::test_ningun_evento_se_edita_ni_se_borra_por_ninguna_ruta. Sin encadenamiento de hashes ni sellado externo; el dueño de la BD puede desactivar el trigger.</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -11154,19 +11290,19 @@
           <t>RF-OPS-001</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>PARCIAL</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1 (avanza)] /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). || Auditoría inicial: Respaldo pg_dump con SHA-256 y simulacro de restauración en BD efímera (app/servicios/respaldo.py:92-205; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella); /api/salud devuelve {'estado':'ok'} sin comprobar BD (app/main.py:84-86); logging.basicConfig a stdout (app/main.py:17); sin métricas; sin healthcheck del servicio web en docker-compose.yml.</t>
+          <t>[Lote 2 (avanza)] Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO. || [Lote 1 (avanza)] /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). || Respaldo pg_dump con SHA-256 y simulacro de restauración en BD efímera (app/servicios/respaldo.py:92-205; tests/test_cierre_pre10.py::test_respaldo_con_simulacro_correcto_y_huella); /api/salud devuelve {'estado':'ok'} sin comprobar BD (app/main.py:84-86); logging.basicConfig a stdout (app/main.py:17); sin métricas; sin healthcheck del servicio web en docker-compose.yml.</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Faltan métricas, health check real (BD, almacenamiento, trabajador) y respaldo de los archivos del almacén (solo segunda copia en el mismo disco). Avance del Lote 1 (avanza): /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). Pendiente: Faltan métricas y el respaldo del almacén fuera del servidor (lote 2).</t>
+          <t>Faltan métricas, health check real (BD, almacenamiento, trabajador) y respaldo de los archivos del almacén (solo segunda copia en el mismo disco). Avance del Lote 1 (avanza): /api/salud revisa base, almacén, latido del trabajador y último respaldo probado (app/servicios/salud.py; tests/test_brechas_lote1.py::test_salud_dice_que_falta_y_solo_la_base_tumba_el_servicio). Pendiente: Faltan métricas y el respaldo del almacén fuera del servidor (lote 2). Avance del Lote 2 (avanza): Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO. Pendiente: Solo faltan métricas.</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Brechas lote 3: HTTPS sin dominio propio, sin caída silenciosa a HTTP, CSP/HSTS y contraseña del administrador respetada
- Despliegue: sin RICORA_DOMINIO usa <ip>.sslip.io para el certificado de
  Let's Encrypt; si el HTTPS falla sigue en HTTP con aviso en el resumen.
- Caddy redirige (302) la dirección numérica al nombre con HTTPS.
- Cabeceras: CSP en todas las respuestas (política propia para /api/docs),
  HSTS solo con HTTPS, Permissions-Policy y COOP.
- Salud: pieza «conexion» degradada si se publica sin HTTPS.
- Interfaz: franja «Conexión sin cifrar» en el ingreso y en cada pantalla.
- La cuenta administradora solo recibe la contraseña del secreto al crearse
  o con RICORA_ADMIN_RESTABLECER=1.
- Corrige «null B» en el tamaño de los originales en papel.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -7459,7 +7459,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>[Lote 1 (avanza)] Segundo factor y auditoría encadenada. || bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
+          <t>[Lote 3 (avanza)] HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts. || [Lote 1 (avanza)] Segundo factor y auditoría encadenada. || bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -7470,7 +7470,7 @@
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Despliegue admite HTTP plano, no hay CSP/HSTS, MFA ni cifrado en reposo, y se envía contenido documental a un servicio externo. Avance del Lote 1 (avanza): Segundo factor y auditoría encadenada. Pendiente: Faltan CSP/HSTS, quitar la caída a HTTP y el restablecimiento de la contraseña del administrador en cada despliegue (lote 3).</t>
+          <t>Despliegue admite HTTP plano, no hay CSP/HSTS, MFA ni cifrado en reposo, y se envía contenido documental a un servicio externo. Avance del Lote 1 (avanza): Segundo factor y auditoría encadenada. Pendiente: Faltan CSP/HSTS, quitar la caída a HTTP y el restablecimiento de la contraseña del administrador en cada despliegue (lote 3). Avance del Lote 3 (avanza): HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts. Pendiente: Pasa a CUMPLE cuando el despliegue confirme el certificado; si el puerto 443 está cerrado en el cortafuegos, hay que abrirlo.</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8259,44 +8259,44 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>NFR-04</t>
+          <t>NFR-01</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>NO EXISTE</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>CUMPLE</t>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 3 (avanza)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
+          <t>HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
+          <t>Pasa a CUMPLE cuando el despliegue confirme el certificado; si el puerto 443 está cerrado en el cortafuegos, hay que abrirlo.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NFR-07</t>
+          <t>NFR-04</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>NO EXISTE</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -8311,19 +8311,19 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
+          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
+          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>RF-OPS-001</t>
+          <t>NFR-07</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -8331,31 +8331,31 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lote 2 (avanza)</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Solo faltan métricas.</t>
+          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>RF-GOV-001</t>
+          <t>RF-OPS-001</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -8363,54 +8363,86 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>NO APLICA</t>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Lote 2 (avanza)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+          <t>Solo faltan métricas.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>RF-GOV-001</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>NFR-05</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>NO CUMPLE</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>NO APLICA</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>Decisión</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor.</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>

</xml_diff>

<commit_message>
Brechas lote 3: NFR-01 confirmado en producción con HTTPS
El despliegue 761aaf4 obtuvo el certificado y respondió por HTTPS con
verificación. Se registra el efecto sobre la base de las URI persistentes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -7452,14 +7452,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>[Lote 3 (avanza)] HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts. || [Lote 1 (avanza)] Segundo factor y auditoría encadenada. || bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
+          <t>[Lote 3] HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts. || [Lote 1 (avanza)] Segundo factor y auditoría encadenada. || bcrypt 12 rondas, JWT HS256 con clave ≥32 obligatoria (app/core/seguridad.py:19-135; app/main.py:20-23), bloqueo por intentos (tests/test_autenticacion.py::test_bloqueo_tras_intentos_fallidos), cabeceras nosniff/DENY (app/main.py:89-95), ClamAV, segunda copia ro. HTTPS opcional con retorno a HTTP y galleta no segura (deploy.yml, RICORA_GALLETA_SEGURA 0); sin CSP/HSTS; secretos en .env plano; sin cifrado en reposo; contraseña admin restablecida en cada despliegue; texto documental enviado a Gemini (app/servicios/motor.py:217).</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -7470,7 +7470,7 @@
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Despliegue admite HTTP plano, no hay CSP/HSTS, MFA ni cifrado en reposo, y se envía contenido documental a un servicio externo. Avance del Lote 1 (avanza): Segundo factor y auditoría encadenada. Pendiente: Faltan CSP/HSTS, quitar la caída a HTTP y el restablecimiento de la contraseña del administrador en cada despliegue (lote 3). Avance del Lote 3 (avanza): HTTPS sin dominio propio (sslip.io + Let's Encrypt con Caddy), sin caída silenciosa a HTTP (aviso en el despliegue, franja en la interfaz y salud «degradado»), CSP y HSTS solo con HTTPS (app/main.py), contraseña del administrador solo al crear o con RICORA_ADMIN_RESTABLECER=1 (app/cli.py); tests/test_brechas_lote3.py, frontend/src/pruebas/sinCifrar.test.ts. Pendiente: Pasa a CUMPLE cuando el despliegue confirme el certificado; si el puerto 443 está cerrado en el cortafuegos, hay que abrirlo.</t>
+          <t>Cerrada en el Lote 3. Riesgo residual: Confirmado en producción (despliegue 761aaf4: HTTPS activo con certificado verificado). Residual: secreto TOTP sin cifrar, estilos en línea en la CSP, nombre prestado (sslip.io) como base de URI persistentes: fijar dominio institucional antes de publicar.</t>
         </is>
       </c>
     </row>
@@ -8267,14 +8267,14 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Lote 3 (avanza)</t>
+          <t>Lote 3</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Pasa a CUMPLE cuando el despliegue confirme el certificado; si el puerto 443 está cerrado en el cortafuegos, hay que abrirlo.</t>
+          <t>Confirmado en producción (despliegue 761aaf4: HTTPS activo con certificado verificado). Residual: secreto TOTP sin cifrar, estilos en línea en la CSP, nombre prestado (sslip.io) como base de URI persistentes: fijar dominio institucional antes de publicar.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Brechas lote 4: buscador unificado de texto completo que respeta la reserva de la Ley 1712
- Migración 0035: configuración ricora_es (español + unaccent), función
  ricora_tsv que recorta un OCR que no quepa en vez de detener la ingesta,
  columnas busqueda con disparadores e índices GIN y de trigramas.
- GET /api/buscar: descripción ISAD(G), texto de los archivos,
  identificadores (código de referencia, VIAF, ORCID…) y autoridades con
  los documentos que las citan; facetas de nivel, años, agente y fondo.
- La búsqueda usa la misma regla de visibilidad del catálogo: el perfil de
  consulta no recibe nada clasificado o reservado ni en fragmentos ni en
  conteos; el equipo de archivo ve además borradores y archivos sin describir.
- Interfaz: caja en la barra superior, página Buscar con fragmentos
  resaltados y por qué coincide cada resultado, y su ayuda.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
@@ -6586,14 +6586,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Solo búsquedas parciales: vocabulario por nombre/trigramas (app/routers/vocabulario.py:143-166), descripciones por título ILIKE (app/routers/descripcion.py:82-89), series (vocabulario.py:217), SPARQL público de solo lectura (app/servicios/sparql.py). No hay búsqueda sobre texto_extraido, alcance, identificadores (codigo_referencia, IdentificadorEntidad) ni índice full-text.</t>
+          <t>[Lote 4] Buscador unificado GET /api/buscar y página Buscar: índice PostgreSQL en español sin tildes (configuración ricora_es, migración 0035) sobre la descripción ISAD(G) y el texto OCR; identificadores (código de referencia, VIAF, ORCID…) completos o por partes; autoridades por nombre y otras formas, con los documentos que las citan; facetas de nivel, años y agente. app/servicios/busqueda.py; tests/test_brechas_lote4.py (palabra solo en el OCR, código de referencia, VIAF). || Solo búsquedas parciales: vocabulario por nombre/trigramas (app/routers/vocabulario.py:143-166), descripciones por título ILIKE (app/routers/descripcion.py:82-89), series (vocabulario.py:217), SPARQL público de solo lectura (app/servicios/sparql.py). No hay búsqueda sobre texto_extraido, alcance, identificadores (codigo_referencia, IdentificadorEntidad) ni índice full-text.</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -6604,7 +6604,7 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>No existe un buscador unificado de texto completo, metadatos, identificadores y contexto.</t>
+          <t>Cerrada en el Lote 4. Riesgo residual: Un OCR de más de ~1 millón de caracteres se indexa recortado; relevancia menos fina que un motor dedicado.</t>
         </is>
       </c>
     </row>
@@ -6639,14 +6639,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Las consultas existentes exigen sesión y módulo (app/core/permisos.py:156-170) y el catálogo/grafo excluye lo reservado (tests/test_grafo_contexto.py::test_el_perfil_de_consulta_no_ve_lo_reservado_en_el_catalogo_ni_en_las_fichas, tests/test_cierre_bloque4_ins.py::test_sparql_responde_sobre_lo_publico_y_no_ve_lo_reservado). Sin buscador general que verificar ni control por fondo.</t>
+          <t>[Lote 4] La búsqueda usa la misma regla de visibilidad del catálogo, RiC-O, grafo e índice (instrumentos.arbol): el perfil de consulta no recibe nada clasificado o reservado, propio o heredado, ni en resultados, fragmentos, conteos ni autoridades; el texto de un archivo reservado no se consulta. tests/test_brechas_lote4.py (3 pruebas de reserva). || Las consultas existentes exigen sesión y módulo (app/core/permisos.py:156-170) y el catálogo/grafo excluye lo reservado (tests/test_grafo_contexto.py::test_el_perfil_de_consulta_no_ve_lo_reservado_en_el_catalogo_ni_en_las_fichas, tests/test_cierre_bloque4_ins.py::test_sparql_responde_sobre_lo_publico_y_no_ve_lo_reservado). Sin buscador general que verificar ni control por fondo.</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -6657,7 +6657,7 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Al no existir búsqueda general ni permisos por fondo, no puede demostrarse que la búsqueda respete restricciones en todos los casos.
+          <t>Cerrada en el Lote 4. Riesgo residual: Sin permisos por fondo y persona (RF-GOV-001 fuera de alcance); las búsquedas no se auditan, por decisión (Ley 1581).
 Perfil AGN: incoherencia si un documento con datos sensibles o de menores queda público.</t>
         </is>
       </c>
@@ -8053,7 +8053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8291,12 +8291,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>NFR-04</t>
+          <t>RF-SEARCH-001</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>NO EXISTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -8306,24 +8306,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 4</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
+          <t>Buscador unificado GET /api/buscar y página Buscar: índice PostgreSQL en español sin tildes (configuración ricora_es, migración 0035) sobre la descripción ISAD(G) y el texto OCR; identificadores (código de referencia, VIAF, ORCID…) completos o por partes; autoridades por nombre y otras formas, con los documentos que las citan; facetas de nivel, años y agente. app/servicios/busqueda.py; tests/test_brechas_lote4.py (palabra solo en el OCR, código de referencia, VIAF).</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
+          <t>Un OCR de más de ~1 millón de caracteres se indexa recortado; relevancia menos fina que un motor dedicado.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>NFR-07</t>
+          <t>RF-SEARCH-002</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -8338,56 +8338,56 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 4</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
+          <t>La búsqueda usa la misma regla de visibilidad del catálogo, RiC-O, grafo e índice (instrumentos.arbol): el perfil de consulta no recibe nada clasificado o reservado, propio o heredado, ni en resultados, fragmentos, conteos ni autoridades; el texto de un archivo reservado no se consulta. tests/test_brechas_lote4.py (3 pruebas de reserva).</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
+          <t>Sin permisos por fondo y persona (RF-GOV-001 fuera de alcance); las búsquedas no se auditan, por decisión (Ley 1581).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>RF-OPS-001</t>
+          <t>NFR-04</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+          <t>NO EXISTE</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Lote 2 (avanza)</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Solo faltan métricas.</t>
+          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>RF-GOV-001</t>
+          <t>NFR-07</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -8395,54 +8395,118 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>NO APLICA</t>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>RF-OPS-001</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Lote 2 (avanza)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Solo faltan métricas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>RF-GOV-001</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t>NFR-05</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>NO CUMPLE</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>NO APLICA</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>Decisión</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>
@@ -10814,26 +10878,22 @@
           <t>RF-SEARCH-001</t>
         </is>
       </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Solo búsquedas parciales: vocabulario por nombre/trigramas (app/routers/vocabulario.py:143-166), descripciones por título ILIKE (app/routers/descripcion.py:82-89), series (vocabulario.py:217), SPARQL público de solo lectura (app/servicios/sparql.py). No hay búsqueda sobre texto_extraido, alcance, identificadores (codigo_referencia, IdentificadorEntidad) ni índice full-text.</t>
+          <t>[Lote 4] Buscador unificado GET /api/buscar y página Buscar: índice PostgreSQL en español sin tildes (configuración ricora_es, migración 0035) sobre la descripción ISAD(G) y el texto OCR; identificadores (código de referencia, VIAF, ORCID…) completos o por partes; autoridades por nombre y otras formas, con los documentos que las citan; facetas de nivel, años y agente. app/servicios/busqueda.py; tests/test_brechas_lote4.py (palabra solo en el OCR, código de referencia, VIAF). || Solo búsquedas parciales: vocabulario por nombre/trigramas (app/routers/vocabulario.py:143-166), descripciones por título ILIKE (app/routers/descripcion.py:82-89), series (vocabulario.py:217), SPARQL público de solo lectura (app/servicios/sparql.py). No hay búsqueda sobre texto_extraido, alcance, identificadores (codigo_referencia, IdentificadorEntidad) ni índice full-text.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>No existe un buscador unificado de texto completo, metadatos, identificadores y contexto.</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Implementar /api/buscar con tsvector/pg_trgm sobre texto OCR, campos ISAD(G), identificadores y nombres alternativos, con facetas por nivel/fecha/agente.</t>
-        </is>
-      </c>
+          <t>Cerrada en el Lote 4. Riesgo residual: Un OCR de más de ~1 millón de caracteres se indexa recortado; relevancia menos fina que un motor dedicado.</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -10857,26 +10917,22 @@
           <t>RF-SEARCH-002</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Las consultas existentes exigen sesión y módulo (app/core/permisos.py:156-170) y el catálogo/grafo excluye lo reservado (tests/test_grafo_contexto.py::test_el_perfil_de_consulta_no_ve_lo_reservado_en_el_catalogo_ni_en_las_fichas, tests/test_cierre_bloque4_ins.py::test_sparql_responde_sobre_lo_publico_y_no_ve_lo_reservado). Sin buscador general que verificar ni control por fondo.</t>
+          <t>[Lote 4] La búsqueda usa la misma regla de visibilidad del catálogo, RiC-O, grafo e índice (instrumentos.arbol): el perfil de consulta no recibe nada clasificado o reservado, propio o heredado, ni en resultados, fragmentos, conteos ni autoridades; el texto de un archivo reservado no se consulta. tests/test_brechas_lote4.py (3 pruebas de reserva). || Las consultas existentes exigen sesión y módulo (app/core/permisos.py:156-170) y el catálogo/grafo excluye lo reservado (tests/test_grafo_contexto.py::test_el_perfil_de_consulta_no_ve_lo_reservado_en_el_catalogo_ni_en_las_fichas, tests/test_cierre_bloque4_ins.py::test_sparql_responde_sobre_lo_publico_y_no_ve_lo_reservado). Sin buscador general que verificar ni control por fondo.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Al no existir búsqueda general ni permisos por fondo, no puede demostrarse que la búsqueda respete restricciones en todos los casos.</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Aplicar el mismo filtro de reserva (derechos.py) y de fondo autorizado dentro del futuro servicio de búsqueda.</t>
-        </is>
-      </c>
+          <t>Cerrada en el Lote 4. Riesgo residual: Sin permisos por fondo y persona (RF-GOV-001 fuera de alcance); las búsquedas no se auditan, por decisión (Ley 1581).</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="inlineStr"/>
       <c r="G25" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Brechas lote 6a: versiones consultables y restaurables de cada descripción y catálogo de atributos con cardinalidad y fuente
- Migración 0037: versiones_descripcion inalterable (huella calculada por la
  base); versión 1 «estado inicial» para lo ya publicado.
- Cada publicación, corrección o restauración crea una versión si algo
  cambió, con atributos y procedencia, contexto, autor, fecha y motivo.
- Historial con cambios (antes → después, fuente) y restauración de los
  atributos de una versión anterior como versión nueva.
- Catálogo de atributos: tipo, cardinalidad, ISAD(G), RiC-O y procedencia;
  validación de cardinalidad con mensaje claro; vista atributo · fuente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -5928,14 +5928,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Crear/consultar/editar: POST /api/descripcion/publicar, GET /api/descripcion/registros/{id}, PATCH /api/descripcion/{id} (app/routers/descripcion.py:246,417,561); vocabulario PATCH /api/vocabulario/{id}. Versionado solo como antes/después JSONB en registro_auditoria (tests/test_descripcion.py::test_reabrir_y_editar_queda_en_auditoria_con_antes_y_despues); RecursoDocumental solo tiene actualizado_en.</t>
+          <t>[Lote 6a] Versiones numeradas e inalterables de cada descripción (migración 0037, versiones_descripcion): instantánea de atributos con procedencia y de contexto, autor, fecha y motivo; historial con cambios; restaurar crea una versión nueva. app/servicios/versiones.py; GET/POST /api/descripcion/registros/{id}/versiones…; tests/test_brechas_lote6.py. || Crear/consultar/editar: POST /api/descripcion/publicar, GET /api/descripcion/registros/{id}, PATCH /api/descripcion/{id} (app/routers/descripcion.py:246,417,561); vocabulario PATCH /api/vocabulario/{id}. Versionado solo como antes/después JSONB en registro_auditoria (tests/test_descripcion.py::test_reabrir_y_editar_queda_en_auditoria_con_antes_y_despues); RecursoDocumental solo tiene actualizado_en.</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -5946,7 +5946,7 @@
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>No hay versiones consultables/restaurables de entidades: el historial depende del log de auditoría.</t>
+          <t>Cerrada en el Lote 6a. Riesgo residual: Restaurar devuelve atributos, no relaciones (cada relación tiene su propia historia de anulación).</t>
         </is>
       </c>
     </row>
@@ -5981,14 +5981,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Atributos como columnas fijas (app/models/recurso_documental.py:47-104); fuente/confianza solo para título, alcance e idiomas (origen_titulo, origen_alcance, confianza_*), y _Procedencia para entidades/relaciones (app/models/descripcion.py:65-78). Perfil de cardinalidades RiC-O documentado: tests/test_ric_o.py::test_el_perfil_de_cardinalidades_esta_escrito_y_documentado.</t>
+          <t>[Lote 6a] Catálogo de atributos (app/servicios/atributos.py): tipo, cardinalidad, ISAD(G), RiC-O y procedencia; validación de cardinalidad al publicar y corregir; vista interna atributo · valor · fuente · confianza. tests/test_brechas_lote6.py. || Atributos como columnas fijas (app/models/recurso_documental.py:47-104); fuente/confianza solo para título, alcance e idiomas (origen_titulo, origen_alcance, confianza_*), y _Procedencia para entidades/relaciones (app/models/descripcion.py:65-78). Perfil de cardinalidades RiC-O documentado: tests/test_ric_o.py::test_el_perfil_de_cardinalidades_esta_escrito_y_documentado.</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -5999,7 +5999,7 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>No hay gestión de atributos (tipo, cardinalidad, fuente) por atributo: el esquema es fijo y la fuente solo existe para algunos campos.
+          <t>Cerrada en el Lote 6a. Riesgo residual: La procedencia de los atributos que el motor no propone se deduce («persona»); autor y fecha en las versiones.
 Perfil AGN: estado de conservación y signatura topográfica del original físico (migración 0031).</t>
         </is>
       </c>
@@ -8053,7 +8053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8419,12 +8419,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>NFR-04</t>
+          <t>RF-RIC-001</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>NO EXISTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -8434,24 +8434,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 6a</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
+          <t>Versiones numeradas e inalterables de cada descripción (migración 0037, versiones_descripcion): instantánea de atributos con procedencia y de contexto, autor, fecha y motivo; historial con cambios; restaurar crea una versión nueva. app/servicios/versiones.py; GET/POST /api/descripcion/registros/{id}/versiones…; tests/test_brechas_lote6.py.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
+          <t>Restaurar devuelve atributos, no relaciones (cada relación tiene su propia historia de anulación).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>NFR-07</t>
+          <t>RF-RIC-002</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -8466,56 +8466,56 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 6a</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
+          <t>Catálogo de atributos (app/servicios/atributos.py): tipo, cardinalidad, ISAD(G), RiC-O y procedencia; validación de cardinalidad al publicar y corregir; vista interna atributo · valor · fuente · confianza. tests/test_brechas_lote6.py.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
+          <t>La procedencia de los atributos que el motor no propone se deduce («persona»); autor y fecha en las versiones.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>RF-OPS-001</t>
+          <t>NFR-04</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+          <t>NO EXISTE</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Lote 2 (avanza)</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Solo faltan métricas.</t>
+          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>RF-GOV-001</t>
+          <t>NFR-07</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -8523,54 +8523,118 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>NO APLICA</t>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>RF-OPS-001</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Lote 2 (avanza)</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Solo faltan métricas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>RF-GOV-001</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>NFR-05</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>NO CUMPLE</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>NO APLICA</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Decisión</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor.</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>
@@ -10539,26 +10603,22 @@
           <t>RF-RIC-001</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Crear/consultar/editar: POST /api/descripcion/publicar, GET /api/descripcion/registros/{id}, PATCH /api/descripcion/{id} (app/routers/descripcion.py:246,417,561); vocabulario PATCH /api/vocabulario/{id}. Versionado solo como antes/después JSONB en registro_auditoria (tests/test_descripcion.py::test_reabrir_y_editar_queda_en_auditoria_con_antes_y_despues); RecursoDocumental solo tiene actualizado_en.</t>
+          <t>[Lote 6a] Versiones numeradas e inalterables de cada descripción (migración 0037, versiones_descripcion): instantánea de atributos con procedencia y de contexto, autor, fecha y motivo; historial con cambios; restaurar crea una versión nueva. app/servicios/versiones.py; GET/POST /api/descripcion/registros/{id}/versiones…; tests/test_brechas_lote6.py. || Crear/consultar/editar: POST /api/descripcion/publicar, GET /api/descripcion/registros/{id}, PATCH /api/descripcion/{id} (app/routers/descripcion.py:246,417,561); vocabulario PATCH /api/vocabulario/{id}. Versionado solo como antes/después JSONB en registro_auditoria (tests/test_descripcion.py::test_reabrir_y_editar_queda_en_auditoria_con_antes_y_despues); RecursoDocumental solo tiene actualizado_en.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>No hay versiones consultables/restaurables de entidades: el historial depende del log de auditoría.</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Crear tablas de versión (o temporal tables) por entidad con número de versión y endpoint GET /versiones y restauración.</t>
-        </is>
-      </c>
+          <t>Cerrada en el Lote 6a. Riesgo residual: Restaurar devuelve atributos, no relaciones (cada relación tiene su propia historia de anulación).</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -10582,26 +10642,22 @@
           <t>RF-RIC-002</t>
         </is>
       </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Atributos como columnas fijas (app/models/recurso_documental.py:47-104); fuente/confianza solo para título, alcance e idiomas (origen_titulo, origen_alcance, confianza_*), y _Procedencia para entidades/relaciones (app/models/descripcion.py:65-78). Perfil de cardinalidades RiC-O documentado: tests/test_ric_o.py::test_el_perfil_de_cardinalidades_esta_escrito_y_documentado.</t>
+          <t>[Lote 6a] Catálogo de atributos (app/servicios/atributos.py): tipo, cardinalidad, ISAD(G), RiC-O y procedencia; validación de cardinalidad al publicar y corregir; vista interna atributo · valor · fuente · confianza. tests/test_brechas_lote6.py. || Atributos como columnas fijas (app/models/recurso_documental.py:47-104); fuente/confianza solo para título, alcance e idiomas (origen_titulo, origen_alcance, confianza_*), y _Procedencia para entidades/relaciones (app/models/descripcion.py:65-78). Perfil de cardinalidades RiC-O documentado: tests/test_ric_o.py::test_el_perfil_de_cardinalidades_esta_escrito_y_documentado.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>No hay gestión de atributos (tipo, cardinalidad, fuente) por atributo: el esquema es fijo y la fuente solo existe para algunos campos.</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Definir un catálogo de atributos con tipo/cardinalidad y registrar procedencia por atributo (o tabla atributo_valor con origen).</t>
-        </is>
-      </c>
+          <t>Cerrada en el Lote 6a. Riesgo residual: La procedencia de los atributos que el motor no propone se deduce («persona»); autor y fecha en las versiones.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Brechas lote 6b: contrato de la API verificado en cada respuesta y versión estable /api/v1
- Las 193 operaciones declaran su respuesta en OpenAPI: esquema JSON
  (modelos en app/schemas/respuestas_*.py, sin filtrar la salida) o el tipo
  de archivo que entregan.
- Prueba de contrato: el cliente de pruebas valida cada respuesta real
  contra el esquema de su ruta; la primera pasada encontró y corrigió 8
  diferencias. Otra prueba exige esquema, resumen y etiqueta en toda ruta.
- /api/v1/… es alias estable de la API y cada respuesta lleva X-API-Version.
- El ingreso documenta sus dos formas: sesión o desafío del segundo factor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DPbqXXn1CAg8rdpv4qL9hL
</commit_message>
<xml_diff>
--- a/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
+++ b/documentacion/RICORA_MATRIZ_MAESTRA_REQUISITOS_v3_0_auditada.xlsx
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -7191,14 +7191,14 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>OpenAPI autogenerado por FastAPI en /api/openapi.json y /api/docs (app/main.py:26-35) con tags y summary para dominio, preservación y auditoría. Muchas rutas devuelven dict sin response_model (p. ej. app/routers/preservacion.py:82-395, app/routers/auditoria.py:56-274) y ningún test valida el contrato OpenAPI.</t>
+          <t>[Lote 6b] Las 193 operaciones (178 rutas) declaran su respuesta en OpenAPI (esquema JSON o tipo de archivo; app/schemas/respuestas_*.py). Prueba de contrato: cada respuesta real de la batería se valida contra el esquema de su ruta (tests/contrato.py, ClienteConContrato); tests/test_contrato_api.py exige esquema, resumen y etiqueta en toda ruta. /api/v1 es alias estable y X-API-Version: 1. || OpenAPI autogenerado por FastAPI en /api/openapi.json y /api/docs (app/main.py:26-35) con tags y summary para dominio, preservación y auditoría. Muchas rutas devuelven dict sin response_model (p. ej. app/routers/preservacion.py:82-395, app/routers/auditoria.py:56-274) y ningún test valida el contrato OpenAPI.</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -7209,7 +7209,7 @@
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>La documentación OpenAPI existe pero con esquemas de respuesta incompletos y sin verificación automática ni versionado de API.</t>
+          <t>Cerrada en el Lote 6b. Riesgo residual: Una ruta que ninguna prueba llama no se valida en ejecución; los campos más variables quedan como objeto genérico.</t>
         </is>
       </c>
     </row>
@@ -8053,7 +8053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8483,12 +8483,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>NFR-04</t>
+          <t>RF-INT-003</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>NO EXISTE</t>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -8498,29 +8498,29 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Lote 2</t>
+          <t>Lote 6b</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
+          <t>Las 193 operaciones (178 rutas) declaran su respuesta en OpenAPI (esquema JSON o tipo de archivo; app/schemas/respuestas_*.py). Prueba de contrato: cada respuesta real de la batería se valida contra el esquema de su ruta (tests/contrato.py, ClienteConContrato); tests/test_contrato_api.py exige esquema, resumen y etiqueta en toda ruta. /api/v1 es alias estable y X-API-Version: 1.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
+          <t>Una ruta que ninguna prueba llama no se valida en ejecución; los campos más variables quedan como objeto genérico.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>NFR-07</t>
+          <t>NFR-04</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PARCIAL</t>
+          <t>NO EXISTE</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
@@ -8535,19 +8535,19 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
+          <t>Cinco escenarios con RPO/RTO objetivo (parámetros) frente a lo medido: app/servicios/recuperacion.py::estado; Preservación › Configuración › Recuperación ante desastres; tests/test_brechas_lote2.py::test_rpo_y_rto_por_escenario_frente_a_lo_medido.</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
+          <t>El tiempo de instalar un servidor nuevo es estimado (2 h), no medido.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>RF-OPS-001</t>
+          <t>NFR-07</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -8555,31 +8555,31 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Lote 2 (avanza)</t>
+          <t>Lote 2</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
+          <t>Paquete de recuperación (base + archivos + manifiesto con huellas, en la misma instantánea) y simulacro integral en base y carpeta nuevas con verificación de filas, huellas y cadena de auditoría; CLI restaurar-paquete; migración 0034; tests/test_brechas_lote2.py.</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Solo faltan métricas.</t>
+          <t>El simulacro corre en el mismo servidor; la restauración en otro servidor se hace con la orden documentada.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>RF-GOV-001</t>
+          <t>RF-OPS-001</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -8587,54 +8587,86 @@
           <t>PARCIAL</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>NO APLICA</t>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Decisión</t>
+          <t>Lote 2 (avanza)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+          <t>Copia completa fuera del servidor: el paquete descargable lleva la base y los archivos; su descarga se registra y mide el RPO.</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+          <t>Solo faltan métricas.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>RF-GOV-001</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>PARCIAL</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>NO APLICA</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Decisión</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Fuera del alcance de la tesis por decisión acordada: varias organizaciones en un mismo sistema no es exigencia del AGN ni aporta al piloto.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Si se despliega para varias entidades, cada una usa su propia instancia (docker-compose).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
           <t>NFR-05</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>NO CUMPLE</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>NO APLICA</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Decisión</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>Fuera del alcance de la tesis por decisión acordada: el piloto corre en un solo servidor.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Para crecer: separar el almacén en un servicio de objetos y varios procesos web.</t>
         </is>
@@ -11354,26 +11386,22 @@
           <t>RF-INT-003</t>
         </is>
       </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>PARCIAL</t>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>OpenAPI autogenerado por FastAPI en /api/openapi.json y /api/docs (app/main.py:26-35) con tags y summary para dominio, preservación y auditoría. Muchas rutas devuelven dict sin response_model (p. ej. app/routers/preservacion.py:82-395, app/routers/auditoria.py:56-274) y ningún test valida el contrato OpenAPI.</t>
+          <t>[Lote 6b] Las 193 operaciones (178 rutas) declaran su respuesta en OpenAPI (esquema JSON o tipo de archivo; app/schemas/respuestas_*.py). Prueba de contrato: cada respuesta real de la batería se valida contra el esquema de su ruta (tests/contrato.py, ClienteConContrato); tests/test_contrato_api.py exige esquema, resumen y etiqueta en toda ruta. /api/v1 es alias estable y X-API-Version: 1. || OpenAPI autogenerado por FastAPI en /api/openapi.json y /api/docs (app/main.py:26-35) con tags y summary para dominio, preservación y auditoría. Muchas rutas devuelven dict sin response_model (p. ej. app/routers/preservacion.py:82-395, app/routers/auditoria.py:56-274) y ningún test valida el contrato OpenAPI.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>La documentación OpenAPI existe pero con esquemas de respuesta incompletos y sin verificación automática ni versionado de API.</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Declarar response_model/ejemplos en todas las rutas, versionar (/api/v1) y añadir prueba que valide openapi.json (p. ej. schemathesis).</t>
-        </is>
-      </c>
+          <t>Cerrada en el Lote 6b. Riesgo residual: Una ruta que ninguna prueba llama no se valida en ejecución; los campos más variables quedan como objeto genérico.</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>

</xml_diff>